<commit_message>
upload dag 19 + aanpassingen dag 17 en dag 18
</commit_message>
<xml_diff>
--- a/Actieplan_Python.xlsx
+++ b/Actieplan_Python.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f020cdb928d38096/Programmeren/Odisee/LevensLang_Leren/LLL-BartBrondeel-2526/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ECD67D8-523A-45D9-ABE9-5625A76A6D1E}"/>
+  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9C55236-F87E-4B83-9568-C9E4BC90B38B}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -755,7 +755,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10">
         <f>('Werkelijke uren'!D32)</f>
-        <v>56.25</v>
+        <v>58.25</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>21</v>
@@ -830,7 +830,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>56.25</v>
+        <v>58.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>56.25</v>
+        <v>58.25</v>
       </c>
     </row>
   </sheetData>
@@ -1315,6 +1315,9 @@
       <c r="B21">
         <v>19</v>
       </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22">
@@ -1372,7 +1375,7 @@
       </c>
       <c r="D32">
         <f>SUM(C3:C32)</f>
-        <v>56.25</v>
+        <v>58.25</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
@@ -1739,7 +1742,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>56.25</v>
+        <v>58.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload dag 20 en 21 + update actieplan
</commit_message>
<xml_diff>
--- a/Actieplan_Python.xlsx
+++ b/Actieplan_Python.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f020cdb928d38096/Programmeren/Odisee/LevensLang_Leren/LLL-BartBrondeel-2526/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9C55236-F87E-4B83-9568-C9E4BC90B38B}"/>
+  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1EAD20B-2581-4E0C-BBD0-50C3CF73D34C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -755,7 +755,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10">
         <f>('Werkelijke uren'!D32)</f>
-        <v>58.25</v>
+        <v>63.25</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>21</v>
@@ -830,7 +830,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>58.25</v>
+        <v>63.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>58.25</v>
+        <v>63.25</v>
       </c>
     </row>
   </sheetData>
@@ -1323,11 +1323,17 @@
       <c r="B22">
         <v>20</v>
       </c>
+      <c r="C22">
+        <v>2</v>
+      </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>21</v>
       </c>
+      <c r="C23">
+        <v>3</v>
+      </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24">
@@ -1375,7 +1381,7 @@
       </c>
       <c r="D32">
         <f>SUM(C3:C32)</f>
-        <v>58.25</v>
+        <v>63.25</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
@@ -1742,7 +1748,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>58.25</v>
+        <v>63.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload dag 22 Pong Game
</commit_message>
<xml_diff>
--- a/Actieplan_Python.xlsx
+++ b/Actieplan_Python.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f020cdb928d38096/Programmeren/Odisee/LevensLang_Leren/LLL-BartBrondeel-2526/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B1EAD20B-2581-4E0C-BBD0-50C3CF73D34C}"/>
+  <xr:revisionPtr revIDLastSave="39" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A56C1EA-5440-4641-8FBA-9DD727488335}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actieplan" sheetId="1" r:id="rId1"/>
@@ -755,7 +755,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10">
         <f>('Werkelijke uren'!D32)</f>
-        <v>63.25</v>
+        <v>65.25</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>21</v>
@@ -830,7 +830,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>63.25</v>
+        <v>65.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>63.25</v>
+        <v>65.25</v>
       </c>
     </row>
   </sheetData>
@@ -1339,6 +1339,9 @@
       <c r="B24">
         <v>22</v>
       </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25">
@@ -1381,7 +1384,7 @@
       </c>
       <c r="D32">
         <f>SUM(C3:C32)</f>
-        <v>63.25</v>
+        <v>65.25</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
@@ -1748,7 +1751,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>63.25</v>
+        <v>65.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload Dag 28 en 29
</commit_message>
<xml_diff>
--- a/Actieplan_Python.xlsx
+++ b/Actieplan_Python.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f020cdb928d38096/Programmeren/Odisee/LevensLang_Leren/LLL-BartBrondeel-2526/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="44" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34C25D81-B0A0-4934-8389-33BDFFAACDBD}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5355F162-99A8-4F3C-B056-5FAE47857C50}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -755,7 +755,7 @@
       <c r="H4" s="10"/>
       <c r="I4" s="10">
         <f>('Werkelijke uren'!D32)</f>
-        <v>77.25</v>
+        <v>83.25</v>
       </c>
       <c r="J4" s="10" t="s">
         <v>21</v>
@@ -830,7 +830,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>77.25</v>
+        <v>83.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>77.25</v>
+        <v>83.25</v>
       </c>
     </row>
   </sheetData>
@@ -1387,11 +1387,17 @@
       <c r="B30">
         <v>28</v>
       </c>
+      <c r="C30">
+        <v>3</v>
+      </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31">
         <v>29</v>
       </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32">
@@ -1399,7 +1405,7 @@
       </c>
       <c r="D32">
         <f>SUM(C3:C32)</f>
-        <v>77.25</v>
+        <v>83.25</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.25">
@@ -1766,7 +1772,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>77.25</v>
+        <v>83.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
upload dag  31 en 32
</commit_message>
<xml_diff>
--- a/Actieplan_Python.xlsx
+++ b/Actieplan_Python.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f020cdb928d38096/Programmeren/Odisee/LevensLang_Leren/LLL-BartBrondeel-2526/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="47" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37309C5F-A0DF-41FD-A4BF-2ACDCDB2A83A}"/>
+  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{900596C3-3D69-4CC9-8CCE-659E9BA1262C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Actieplan" sheetId="1" r:id="rId1"/>
@@ -784,7 +784,7 @@
       <c r="H5" s="10"/>
       <c r="I5" s="10">
         <f>('Werkelijke uren'!D62)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>22</v>
@@ -830,7 +830,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>85.25</v>
+        <v>90.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>85.25</v>
+        <v>90.25</v>
       </c>
     </row>
   </sheetData>
@@ -1411,82 +1411,88 @@
         <v>85.25</v>
       </c>
     </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B33">
         <v>31</v>
       </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C33">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="34" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B34">
         <v>32</v>
       </c>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="C34">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B35">
         <v>33</v>
       </c>
     </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
         <v>35</v>
       </c>
     </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B38">
         <v>36</v>
       </c>
     </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B39">
         <v>37</v>
       </c>
     </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B40">
         <v>38</v>
       </c>
     </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B41">
         <v>39</v>
       </c>
     </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B42">
         <v>40</v>
       </c>
     </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B43">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B44">
         <v>42</v>
       </c>
     </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B45">
         <v>43</v>
       </c>
     </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B46">
         <v>44</v>
       </c>
     </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B47">
         <v>45</v>
       </c>
     </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B48">
         <v>46</v>
       </c>
@@ -1562,7 +1568,7 @@
       </c>
       <c r="D62">
         <f>SUM(C33:C62)</f>
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.25">
@@ -1775,7 +1781,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>85.25</v>
+        <v>90.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Upload dag 33 en 34
</commit_message>
<xml_diff>
--- a/Actieplan_Python.xlsx
+++ b/Actieplan_Python.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f020cdb928d38096/Programmeren/Odisee/LevensLang_Leren/LLL-BartBrondeel-2526/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="49" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{900596C3-3D69-4CC9-8CCE-659E9BA1262C}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="13_ncr:1_{482E40B1-4C12-41F6-8D36-DD9DCD6004AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16586C5A-377B-42EF-86B9-3379F31DD4B2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -784,7 +784,7 @@
       <c r="H5" s="10"/>
       <c r="I5" s="10">
         <f>('Werkelijke uren'!D62)</f>
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="J5" s="10" t="s">
         <v>22</v>
@@ -830,7 +830,7 @@
       <c r="H7" s="10"/>
       <c r="I7" s="10">
         <f>('Werkelijke uren'!C103)</f>
-        <v>90.25</v>
+        <v>96.25</v>
       </c>
       <c r="J7" s="10"/>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="I22">
         <f>SUM(I7,I14,I20)</f>
-        <v>90.25</v>
+        <v>96.25</v>
       </c>
     </row>
   </sheetData>
@@ -1431,11 +1431,17 @@
       <c r="B35">
         <v>33</v>
       </c>
+      <c r="C35">
+        <v>3</v>
+      </c>
     </row>
     <row r="36" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B36">
         <v>34</v>
       </c>
+      <c r="C36">
+        <v>3</v>
+      </c>
     </row>
     <row r="37" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B37">
@@ -1568,7 +1574,7 @@
       </c>
       <c r="D62">
         <f>SUM(C33:C62)</f>
-        <v>5</v>
+        <v>11</v>
       </c>
     </row>
     <row r="63" spans="2:4" x14ac:dyDescent="0.25">
@@ -1781,7 +1787,7 @@
       </c>
       <c r="C103">
         <f>SUM(C3:C102)</f>
-        <v>90.25</v>
+        <v>96.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>